<commit_message>
Auto-analysis: mbb — 2026-08-30
</commit_message>
<xml_diff>
--- a/Bao cao/MBB/MBB_Model_2026_08_30.xlsx
+++ b/Bao cao/MBB/MBB_Model_2026_08_30.xlsx
@@ -27,6 +27,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_PE_PB_History" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Credit_Funding_Growth" sheetId="19" state="visible" r:id="rId19"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Peer_Benchmark" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_ALM_LaiSuat_ThanhKhoan" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -41,7 +42,7 @@
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="0.0"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -128,6 +129,11 @@
       <i val="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="13"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -185,7 +191,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -241,6 +247,11 @@
     <xf numFmtId="10" fontId="1" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="1" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="1" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -12475,13 +12486,13 @@
         <v>0.14</v>
       </c>
       <c r="B6" s="20" t="n">
-        <v>41567.62958507127</v>
+        <v>41567.62958507126</v>
       </c>
       <c r="C6" s="30" t="n">
-        <v>43252.76950750897</v>
+        <v>43252.76950750896</v>
       </c>
       <c r="D6" s="30" t="n">
-        <v>45244.29850675351</v>
+        <v>45244.2985067535</v>
       </c>
       <c r="E6" s="20" t="n">
         <v>47634.13330584698</v>
@@ -14605,7 +14616,7 @@
         <v>16.70611111111111</v>
       </c>
       <c r="E2" s="38" t="n">
-        <v>16.47333333333333</v>
+        <v>16.47333333333334</v>
       </c>
       <c r="F2" s="38" t="n">
         <v>32.68222222222222</v>
@@ -14614,7 +14625,7 @@
         <v>1.384444444444445</v>
       </c>
       <c r="H2" s="38" t="n">
-        <v>5.505</v>
+        <v>5.504999999999999</v>
       </c>
       <c r="I2" s="37" t="inlineStr">
         <is>
@@ -15181,6 +15192,79 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="45" t="inlineStr">
+        <is>
+          <t>PHÂN TÍCH RỦI RO LÃI SUẤT &amp; THANH KHOẢN (ALM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Nguồn: Báo cáo tài chính hợp nhất quý 2 năm 2026 (đã soát xét) (năm 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/MBB_202608062020MBB2020BCTC20hop20nhat20soat20xet20ban20nien202026_10082026095318.pdf?v=1786330399877</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>TÓM TẮT</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="46" t="inlineStr">
+        <is>
+          <t>Rủi ro lãi suất: mức tham chiếu Đáng chú ý (gap +12.61% tổng tài sản), khả năng chống chịu VỪA PHẢI — NII biến động đáng kể nhưng chưa ở mức nghiêm trọng (kịch bản sốc mạnh nhất làm NII đổi khoảng 6.8%). Rủi ro thanh khoản: mức tham chiếu Trung bình, khả năng chống chịu TỐT — tài sản thanh khoản đủ bù ngay cả kịch bản rút tiền gửi mạnh nhất đã test (che phủ 139% ở kịch bản rút tiền gửi mạnh nhất).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="10">
+      <c r="A10" s="47" t="inlineStr">
+        <is>
+          <t>A. RỦI RO LÃI SUẤT — Khe hở nhạy cảm lãi suất theo kỳ hạn</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A6:J8"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -15211,7 +15295,7 @@
     <row r="4">
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>Ngày lập: 30/08/2026 18:40</t>
+          <t>Ngày lập: 30/08/2026 22:35</t>
         </is>
       </c>
     </row>

</xml_diff>